<commit_message>
Fix notebook bugs and re-run all LR estimation pipelines
- Fix np.trapz -> np.trapezoid deprecation in compare_lr_estimates
- Guard reasoning param for non-o-series models in estimate_differential_lrs
- Fix verbosity "low" -> "medium" for gpt-4.1-nano compatibility
- Fix dtype handling for DataFrame column assignment
- Re-run all 4 notebooks with gpt-4.1-nano-2025-04-14, update output xlsx/pdf

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/archive/legacy_runs/lr_estimation_2025_07_21/LRs for 87 features within GI ddx - dysphagia vs esophageal pain without dysphagia_filled.xlsx
+++ b/archive/legacy_runs/lr_estimation_2025_07_21/LRs for 87 features within GI ddx - dysphagia vs esophageal pain without dysphagia_filled.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -446,7 +446,7 @@
       <c r="S1" t="inlineStr"/>
       <c r="T1" t="inlineStr">
         <is>
-          <t>Differential LR (gpt-5-mini for 'Pain Due to Esophageal Dysphagia' vs. 'Esophageal discomfort without dysphagia')</t>
+          <t>Differential LR (gpt-4.1-nano-2025-04-14 for 'Pain Due to Esophageal Dysphagia' vs. 'Esophageal discomfort without dysphagia')</t>
         </is>
       </c>
     </row>
@@ -569,7 +569,7 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -597,7 +597,7 @@
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
-        <v>2.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -625,7 +625,7 @@
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
-        <v>8</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="6">
@@ -653,7 +653,7 @@
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="n">
-        <v>3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
@@ -681,7 +681,7 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
-        <v>5.2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="8">
@@ -709,7 +709,7 @@
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="9">
@@ -737,7 +737,7 @@
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
-        <v>0.33</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="10">
@@ -765,7 +765,7 @@
       <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="11">
@@ -793,7 +793,7 @@
       <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="n">
-        <v>0.29</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="12">
@@ -821,7 +821,7 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="13">
@@ -849,7 +849,7 @@
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="n">
-        <v>2.7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
@@ -877,7 +877,7 @@
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15">
@@ -905,7 +905,7 @@
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16">
@@ -933,7 +933,7 @@
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
@@ -961,7 +961,7 @@
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="n">
-        <v>3.3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
@@ -989,7 +989,7 @@
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="n">
-        <v>1.3</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="19">
@@ -1017,7 +1017,7 @@
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="n">
-        <v>1.3</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="20">
@@ -1045,7 +1045,7 @@
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="n">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="21">
@@ -1073,7 +1073,7 @@
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="n">
-        <v>2.7</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="22">
@@ -1101,7 +1101,7 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="n">
-        <v>1.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="23">
@@ -1129,7 +1129,7 @@
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="n">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="24">
@@ -1157,7 +1157,7 @@
       <c r="R24" t="inlineStr"/>
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="n">
-        <v>0.96</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="25">
@@ -1185,7 +1185,7 @@
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="26">
@@ -1213,7 +1213,7 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="n">
-        <v>0.96</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="27">
@@ -1241,7 +1241,7 @@
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="n">
-        <v>0.43</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="28">
@@ -1269,7 +1269,7 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="n">
-        <v>1.7</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="29">
@@ -1297,7 +1297,7 @@
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="30">
@@ -1325,7 +1325,7 @@
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31">
@@ -1381,7 +1381,7 @@
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="n">
-        <v>0.33</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="33">
@@ -1409,7 +1409,7 @@
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="34">
@@ -1437,7 +1437,7 @@
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="n">
-        <v>0.3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
@@ -1465,7 +1465,7 @@
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36">
@@ -1493,7 +1493,7 @@
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="37">
@@ -1521,7 +1521,7 @@
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="38">
@@ -1549,7 +1549,7 @@
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="n">
-        <v>1.2</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="39">
@@ -1577,7 +1577,7 @@
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="n">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="40">
@@ -1605,7 +1605,7 @@
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="n">
-        <v>1.4</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="41">
@@ -1633,7 +1633,7 @@
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="n">
-        <v>0.8</v>
+        <v>0.083</v>
       </c>
     </row>
     <row r="42">
@@ -1661,7 +1661,7 @@
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="43">
@@ -1689,7 +1689,7 @@
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="44">
@@ -1717,7 +1717,7 @@
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="45">
@@ -1745,7 +1745,7 @@
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="46">
@@ -1773,7 +1773,7 @@
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="n">
-        <v>1.2</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="47">
@@ -1801,7 +1801,7 @@
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="n">
-        <v>1.4</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="48">
@@ -1829,7 +1829,7 @@
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="49">
@@ -1857,7 +1857,7 @@
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="50">
@@ -1885,7 +1885,7 @@
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="51">
@@ -1913,7 +1913,7 @@
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="52">
@@ -1941,7 +1941,7 @@
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="n">
-        <v>0.95</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="53">
@@ -1969,7 +1969,7 @@
       <c r="R53" t="inlineStr"/>
       <c r="S53" t="inlineStr"/>
       <c r="T53" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="54">
@@ -1997,7 +1997,7 @@
       <c r="R54" t="inlineStr"/>
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="55">
@@ -2025,7 +2025,7 @@
       <c r="R55" t="inlineStr"/>
       <c r="S55" t="inlineStr"/>
       <c r="T55" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -2053,7 +2053,7 @@
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="57">
@@ -2081,7 +2081,7 @@
       <c r="R57" t="inlineStr"/>
       <c r="S57" t="inlineStr"/>
       <c r="T57" t="n">
-        <v>1.5</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="58">
@@ -2109,7 +2109,7 @@
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="59">
@@ -2137,7 +2137,7 @@
       <c r="R59" t="inlineStr"/>
       <c r="S59" t="inlineStr"/>
       <c r="T59" t="n">
-        <v>0.9</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="60">
@@ -2165,7 +2165,7 @@
       <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="61">
@@ -2193,7 +2193,7 @@
       <c r="R61" t="inlineStr"/>
       <c r="S61" t="inlineStr"/>
       <c r="T61" t="n">
-        <v>1.4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="62">
@@ -2221,7 +2221,7 @@
       <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="n">
-        <v>1.4</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="63">
@@ -2249,7 +2249,7 @@
       <c r="R63" t="inlineStr"/>
       <c r="S63" t="inlineStr"/>
       <c r="T63" t="n">
-        <v>1</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="64">
@@ -2277,7 +2277,7 @@
       <c r="R64" t="inlineStr"/>
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="65">
@@ -2305,7 +2305,7 @@
       <c r="R65" t="inlineStr"/>
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="n">
-        <v>1.06</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="66">
@@ -2333,7 +2333,7 @@
       <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr"/>
       <c r="T66" t="n">
-        <v>1.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="67">
@@ -2389,7 +2389,7 @@
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr"/>
       <c r="T68" t="n">
-        <v>0.82</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="69">
@@ -2417,7 +2417,7 @@
       <c r="R69" t="inlineStr"/>
       <c r="S69" t="inlineStr"/>
       <c r="T69" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="70">
@@ -2445,7 +2445,7 @@
       <c r="R70" t="inlineStr"/>
       <c r="S70" t="inlineStr"/>
       <c r="T70" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="71">
@@ -2473,7 +2473,7 @@
       <c r="R71" t="inlineStr"/>
       <c r="S71" t="inlineStr"/>
       <c r="T71" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="72">
@@ -2501,7 +2501,7 @@
       <c r="R72" t="inlineStr"/>
       <c r="S72" t="inlineStr"/>
       <c r="T72" t="n">
-        <v>1.03</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="73">
@@ -2529,7 +2529,7 @@
       <c r="R73" t="inlineStr"/>
       <c r="S73" t="inlineStr"/>
       <c r="T73" t="n">
-        <v>0.82</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="74">
@@ -2557,7 +2557,7 @@
       <c r="R74" t="inlineStr"/>
       <c r="S74" t="inlineStr"/>
       <c r="T74" t="n">
-        <v>1.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="75">
@@ -2585,7 +2585,7 @@
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="inlineStr"/>
       <c r="T75" t="n">
-        <v>1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="76">
@@ -2613,7 +2613,7 @@
       <c r="R76" t="inlineStr"/>
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="77">
@@ -2641,7 +2641,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>0.8</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="78">
@@ -2669,7 +2669,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr"/>
       <c r="T78" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="79">
@@ -2697,7 +2697,7 @@
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>0.97</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="80">
@@ -2725,7 +2725,7 @@
       <c r="R80" t="inlineStr"/>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="81">
@@ -2753,7 +2753,7 @@
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="82">
@@ -2781,7 +2781,7 @@
       <c r="R82" t="inlineStr"/>
       <c r="S82" t="inlineStr"/>
       <c r="T82" t="n">
-        <v>0.95</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="83">
@@ -2809,7 +2809,7 @@
       <c r="R83" t="inlineStr"/>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="84">
@@ -2837,7 +2837,7 @@
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="inlineStr"/>
       <c r="T84" t="n">
-        <v>1.1</v>
+        <v>0.33</v>
       </c>
     </row>
     <row r="85">
@@ -2865,7 +2865,7 @@
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="inlineStr"/>
       <c r="T85" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="86">
@@ -2893,7 +2893,7 @@
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="inlineStr"/>
       <c r="T86" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="87">
@@ -2921,7 +2921,7 @@
       <c r="R87" t="inlineStr"/>
       <c r="S87" t="inlineStr"/>
       <c r="T87" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="88">
@@ -2949,7 +2949,7 @@
       <c r="R88" t="inlineStr"/>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>1.02</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="89">
@@ -2977,7 +2977,7 @@
       <c r="R89" t="inlineStr"/>
       <c r="S89" t="inlineStr"/>
       <c r="T89" t="n">
-        <v>1.06</v>
+        <v>0.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Document notebook manifest logic
</commit_message>
<xml_diff>
--- a/archive/legacy_runs/lr_estimation_2025_07_21/LRs for 87 features within GI ddx - dysphagia vs esophageal pain without dysphagia_filled.xlsx
+++ b/archive/legacy_runs/lr_estimation_2025_07_21/LRs for 87 features within GI ddx - dysphagia vs esophageal pain without dysphagia_filled.xlsx
@@ -569,7 +569,7 @@
       <c r="R3" t="inlineStr"/>
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -597,7 +597,7 @@
       <c r="R4" t="inlineStr"/>
       <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
-        <v>8</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="5">
@@ -625,7 +625,7 @@
       <c r="R5" t="inlineStr"/>
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="6">
@@ -653,7 +653,7 @@
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="7">
@@ -681,7 +681,7 @@
       <c r="R7" t="inlineStr"/>
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="8">
@@ -709,7 +709,7 @@
       <c r="R8" t="inlineStr"/>
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="n">
-        <v>0.3</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="9">
@@ -737,7 +737,7 @@
       <c r="R9" t="inlineStr"/>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10">
@@ -821,7 +821,7 @@
       <c r="R12" t="inlineStr"/>
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="13">
@@ -849,7 +849,7 @@
       <c r="R13" t="inlineStr"/>
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="n">
-        <v>4</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="14">
@@ -877,7 +877,7 @@
       <c r="R14" t="inlineStr"/>
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
@@ -905,7 +905,7 @@
       <c r="R15" t="inlineStr"/>
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
@@ -961,7 +961,7 @@
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="inlineStr"/>
       <c r="T17" t="n">
-        <v>2</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="18">
@@ -989,7 +989,7 @@
       <c r="R18" t="inlineStr"/>
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="n">
-        <v>0.33</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="19">
@@ -1017,7 +1017,7 @@
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="20">
@@ -1045,7 +1045,7 @@
       <c r="R20" t="inlineStr"/>
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="21">
@@ -1073,7 +1073,7 @@
       <c r="R21" t="inlineStr"/>
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="22">
@@ -1101,7 +1101,7 @@
       <c r="R22" t="inlineStr"/>
       <c r="S22" t="inlineStr"/>
       <c r="T22" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="23">
@@ -1129,7 +1129,7 @@
       <c r="R23" t="inlineStr"/>
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="24">
@@ -1185,7 +1185,7 @@
       <c r="R25" t="inlineStr"/>
       <c r="S25" t="inlineStr"/>
       <c r="T25" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="26">
@@ -1213,7 +1213,7 @@
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="inlineStr"/>
       <c r="T26" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="27">
@@ -1241,7 +1241,7 @@
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="inlineStr"/>
       <c r="T27" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="28">
@@ -1269,7 +1269,7 @@
       <c r="R28" t="inlineStr"/>
       <c r="S28" t="inlineStr"/>
       <c r="T28" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="29">
@@ -1297,7 +1297,7 @@
       <c r="R29" t="inlineStr"/>
       <c r="S29" t="inlineStr"/>
       <c r="T29" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -1325,7 +1325,7 @@
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="inlineStr"/>
       <c r="T30" t="n">
-        <v>15</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="31">
@@ -1353,7 +1353,7 @@
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
       <c r="T31" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
@@ -1381,7 +1381,7 @@
       <c r="R32" t="inlineStr"/>
       <c r="S32" t="inlineStr"/>
       <c r="T32" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="33">
@@ -1409,7 +1409,7 @@
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="inlineStr"/>
       <c r="T33" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="34">
@@ -1437,7 +1437,7 @@
       <c r="R34" t="inlineStr"/>
       <c r="S34" t="inlineStr"/>
       <c r="T34" t="n">
-        <v>4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="35">
@@ -1465,7 +1465,7 @@
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
       <c r="T35" t="n">
-        <v>8</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="36">
@@ -1493,7 +1493,7 @@
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
       <c r="T36" t="n">
-        <v>0.15</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="37">
@@ -1521,7 +1521,7 @@
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
       <c r="T37" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="38">
@@ -1549,7 +1549,7 @@
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
       <c r="T38" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -1577,7 +1577,7 @@
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="inlineStr"/>
       <c r="T39" t="n">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="40">
@@ -1605,7 +1605,7 @@
       <c r="R40" t="inlineStr"/>
       <c r="S40" t="inlineStr"/>
       <c r="T40" t="n">
-        <v>0.2</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="41">
@@ -1633,7 +1633,7 @@
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="inlineStr"/>
       <c r="T41" t="n">
-        <v>0.083</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="42">
@@ -1661,7 +1661,7 @@
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="inlineStr"/>
       <c r="T42" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
@@ -1689,7 +1689,7 @@
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr"/>
       <c r="T43" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="44">
@@ -1717,7 +1717,7 @@
       <c r="R44" t="inlineStr"/>
       <c r="S44" t="inlineStr"/>
       <c r="T44" t="n">
-        <v>0.8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -1745,7 +1745,7 @@
       <c r="R45" t="inlineStr"/>
       <c r="S45" t="inlineStr"/>
       <c r="T45" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="46">
@@ -1773,7 +1773,7 @@
       <c r="R46" t="inlineStr"/>
       <c r="S46" t="inlineStr"/>
       <c r="T46" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="47">
@@ -1801,7 +1801,7 @@
       <c r="R47" t="inlineStr"/>
       <c r="S47" t="inlineStr"/>
       <c r="T47" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="48">
@@ -1829,7 +1829,7 @@
       <c r="R48" t="inlineStr"/>
       <c r="S48" t="inlineStr"/>
       <c r="T48" t="n">
-        <v>0.4</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="49">
@@ -1857,7 +1857,7 @@
       <c r="R49" t="inlineStr"/>
       <c r="S49" t="inlineStr"/>
       <c r="T49" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="50">
@@ -1885,7 +1885,7 @@
       <c r="R50" t="inlineStr"/>
       <c r="S50" t="inlineStr"/>
       <c r="T50" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="51">
@@ -1913,7 +1913,7 @@
       <c r="R51" t="inlineStr"/>
       <c r="S51" t="inlineStr"/>
       <c r="T51" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="52">
@@ -1941,7 +1941,7 @@
       <c r="R52" t="inlineStr"/>
       <c r="S52" t="inlineStr"/>
       <c r="T52" t="n">
-        <v>0.15</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="53">
@@ -1969,7 +1969,7 @@
       <c r="R53" t="inlineStr"/>
       <c r="S53" t="inlineStr"/>
       <c r="T53" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="54">
@@ -1997,7 +1997,7 @@
       <c r="R54" t="inlineStr"/>
       <c r="S54" t="inlineStr"/>
       <c r="T54" t="n">
-        <v>0.4</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="55">
@@ -2025,7 +2025,7 @@
       <c r="R55" t="inlineStr"/>
       <c r="S55" t="inlineStr"/>
       <c r="T55" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="56">
@@ -2053,7 +2053,7 @@
       <c r="R56" t="inlineStr"/>
       <c r="S56" t="inlineStr"/>
       <c r="T56" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="57">
@@ -2081,7 +2081,7 @@
       <c r="R57" t="inlineStr"/>
       <c r="S57" t="inlineStr"/>
       <c r="T57" t="n">
-        <v>0.67</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="58">
@@ -2109,7 +2109,7 @@
       <c r="R58" t="inlineStr"/>
       <c r="S58" t="inlineStr"/>
       <c r="T58" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="59">
@@ -2137,7 +2137,7 @@
       <c r="R59" t="inlineStr"/>
       <c r="S59" t="inlineStr"/>
       <c r="T59" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60">
@@ -2165,7 +2165,7 @@
       <c r="R60" t="inlineStr"/>
       <c r="S60" t="inlineStr"/>
       <c r="T60" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="61">
@@ -2221,7 +2221,7 @@
       <c r="R62" t="inlineStr"/>
       <c r="S62" t="inlineStr"/>
       <c r="T62" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="63">
@@ -2249,7 +2249,7 @@
       <c r="R63" t="inlineStr"/>
       <c r="S63" t="inlineStr"/>
       <c r="T63" t="n">
-        <v>0.4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64">
@@ -2277,7 +2277,7 @@
       <c r="R64" t="inlineStr"/>
       <c r="S64" t="inlineStr"/>
       <c r="T64" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="65">
@@ -2305,7 +2305,7 @@
       <c r="R65" t="inlineStr"/>
       <c r="S65" t="inlineStr"/>
       <c r="T65" t="n">
-        <v>0.5</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="66">
@@ -2333,7 +2333,7 @@
       <c r="R66" t="inlineStr"/>
       <c r="S66" t="inlineStr"/>
       <c r="T66" t="n">
-        <v>0.8</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="67">
@@ -2389,7 +2389,7 @@
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr"/>
       <c r="T68" t="n">
-        <v>0.33</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -2417,7 +2417,7 @@
       <c r="R69" t="inlineStr"/>
       <c r="S69" t="inlineStr"/>
       <c r="T69" t="n">
-        <v>0.3</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="70">
@@ -2445,7 +2445,7 @@
       <c r="R70" t="inlineStr"/>
       <c r="S70" t="inlineStr"/>
       <c r="T70" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="71">
@@ -2501,7 +2501,7 @@
       <c r="R72" t="inlineStr"/>
       <c r="S72" t="inlineStr"/>
       <c r="T72" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="73">
@@ -2529,7 +2529,7 @@
       <c r="R73" t="inlineStr"/>
       <c r="S73" t="inlineStr"/>
       <c r="T73" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="74">
@@ -2557,7 +2557,7 @@
       <c r="R74" t="inlineStr"/>
       <c r="S74" t="inlineStr"/>
       <c r="T74" t="n">
-        <v>0.2</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="75">
@@ -2585,7 +2585,7 @@
       <c r="R75" t="inlineStr"/>
       <c r="S75" t="inlineStr"/>
       <c r="T75" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="76">
@@ -2613,7 +2613,7 @@
       <c r="R76" t="inlineStr"/>
       <c r="S76" t="inlineStr"/>
       <c r="T76" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="77">
@@ -2641,7 +2641,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr"/>
       <c r="T77" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="78">
@@ -2669,7 +2669,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr"/>
       <c r="T78" t="n">
-        <v>0.3</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="79">
@@ -2697,7 +2697,7 @@
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="inlineStr"/>
       <c r="T79" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="80">
@@ -2725,7 +2725,7 @@
       <c r="R80" t="inlineStr"/>
       <c r="S80" t="inlineStr"/>
       <c r="T80" t="n">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="81">
@@ -2753,7 +2753,7 @@
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="inlineStr"/>
       <c r="T81" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="82">
@@ -2781,7 +2781,7 @@
       <c r="R82" t="inlineStr"/>
       <c r="S82" t="inlineStr"/>
       <c r="T82" t="n">
-        <v>0.3</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="83">
@@ -2809,7 +2809,7 @@
       <c r="R83" t="inlineStr"/>
       <c r="S83" t="inlineStr"/>
       <c r="T83" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="84">
@@ -2837,7 +2837,7 @@
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="inlineStr"/>
       <c r="T84" t="n">
-        <v>0.33</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="85">
@@ -2865,7 +2865,7 @@
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="inlineStr"/>
       <c r="T85" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="86">
@@ -2893,7 +2893,7 @@
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="inlineStr"/>
       <c r="T86" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="87">
@@ -2949,7 +2949,7 @@
       <c r="R88" t="inlineStr"/>
       <c r="S88" t="inlineStr"/>
       <c r="T88" t="n">
-        <v>0.05</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="89">
@@ -2977,7 +2977,7 @@
       <c r="R89" t="inlineStr"/>
       <c r="S89" t="inlineStr"/>
       <c r="T89" t="n">
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>